<commit_message>
Fixed bug where branch prediction stalls were resolved prematurely in the decode stage.
</commit_message>
<xml_diff>
--- a/project/outputs_xlsx_solution/test33.1-wide.xlsx
+++ b/project/outputs_xlsx_solution/test33.1-wide.xlsx
@@ -990,6 +990,12 @@
       <c r="EJ1">
         <v>137</v>
       </c>
+      <c r="EK1">
+        <v>138</v>
+      </c>
+      <c r="EL1">
+        <v>139</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2">
@@ -2166,6 +2172,9 @@
       <c r="AV40" t="s">
         <v>5</v>
       </c>
+      <c r="AW40" t="s">
+        <v>6</v>
+      </c>
       <c r="AX40" t="s">
         <v>8</v>
       </c>
@@ -2186,17 +2195,11 @@
       <c r="C41" t="s">
         <v>18</v>
       </c>
-      <c r="AW41" t="s">
-        <v>5</v>
-      </c>
-      <c r="AX41" t="s">
-        <v>6</v>
-      </c>
       <c r="AY41" t="s">
-        <v>32</v>
+        <v>5</v>
       </c>
       <c r="AZ41" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="BA41" t="s">
         <v>8</v>
@@ -2205,6 +2208,9 @@
         <v>8</v>
       </c>
       <c r="BC41" t="s">
+        <v>8</v>
+      </c>
+      <c r="BD41" t="s">
         <v>10</v>
       </c>
       <c r="BI41" t="s">
@@ -2221,18 +2227,15 @@
       <c r="C42" t="s">
         <v>19</v>
       </c>
-      <c r="AX42" t="s">
-        <v>5</v>
-      </c>
-      <c r="AY42" t="s">
-        <v>6</v>
-      </c>
       <c r="AZ42" t="s">
+        <v>5</v>
+      </c>
+      <c r="BA42" t="s">
+        <v>6</v>
+      </c>
+      <c r="BB42" t="s">
         <v>21</v>
       </c>
-      <c r="BC42" t="s">
-        <v>8</v>
-      </c>
       <c r="BD42" t="s">
         <v>8</v>
       </c>
@@ -2240,7 +2243,7 @@
         <v>8</v>
       </c>
       <c r="BF42" t="s">
-        <v>26</v>
+        <v>8</v>
       </c>
       <c r="BG42" t="s">
         <v>26</v>
@@ -2249,9 +2252,12 @@
         <v>26</v>
       </c>
       <c r="BI42" t="s">
-        <v>10</v>
+        <v>26</v>
       </c>
       <c r="BJ42" t="s">
+        <v>26</v>
+      </c>
+      <c r="BK42" t="s">
         <v>11</v>
       </c>
     </row>
@@ -2265,24 +2271,18 @@
       <c r="C43" t="s">
         <v>20</v>
       </c>
-      <c r="AY43" t="s">
-        <v>5</v>
-      </c>
-      <c r="AZ43" t="s">
-        <v>6</v>
-      </c>
       <c r="BA43" t="s">
+        <v>5</v>
+      </c>
+      <c r="BB43" t="s">
+        <v>6</v>
+      </c>
+      <c r="BC43" t="s">
         <v>21</v>
       </c>
-      <c r="BI43" t="s">
+      <c r="BK43" t="s">
         <v>32</v>
       </c>
-      <c r="BJ43" t="s">
-        <v>8</v>
-      </c>
-      <c r="BK43" t="s">
-        <v>8</v>
-      </c>
       <c r="BL43" t="s">
         <v>8</v>
       </c>
@@ -2290,9 +2290,15 @@
         <v>8</v>
       </c>
       <c r="BN43" t="s">
-        <v>26</v>
+        <v>8</v>
       </c>
       <c r="BO43" t="s">
+        <v>8</v>
+      </c>
+      <c r="BP43" t="s">
+        <v>26</v>
+      </c>
+      <c r="BQ43" t="s">
         <v>11</v>
       </c>
     </row>
@@ -2306,17 +2312,11 @@
       <c r="C44" t="s">
         <v>22</v>
       </c>
-      <c r="AZ44" t="s">
-        <v>5</v>
-      </c>
-      <c r="BA44" t="s">
-        <v>6</v>
-      </c>
       <c r="BB44" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="BC44" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="BD44" t="s">
         <v>8</v>
@@ -2325,10 +2325,10 @@
         <v>8</v>
       </c>
       <c r="BF44" t="s">
-        <v>26</v>
+        <v>8</v>
       </c>
       <c r="BG44" t="s">
-        <v>26</v>
+        <v>8</v>
       </c>
       <c r="BH44" t="s">
         <v>26</v>
@@ -2337,9 +2337,15 @@
         <v>26</v>
       </c>
       <c r="BJ44" t="s">
-        <v>10</v>
-      </c>
-      <c r="BP44" t="s">
+        <v>26</v>
+      </c>
+      <c r="BK44" t="s">
+        <v>26</v>
+      </c>
+      <c r="BL44" t="s">
+        <v>10</v>
+      </c>
+      <c r="BR44" t="s">
         <v>11</v>
       </c>
     </row>
@@ -2353,17 +2359,11 @@
       <c r="C45" t="s">
         <v>23</v>
       </c>
-      <c r="BA45" t="s">
-        <v>5</v>
-      </c>
-      <c r="BB45" t="s">
-        <v>6</v>
-      </c>
       <c r="BC45" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="BD45" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="BE45" t="s">
         <v>8</v>
@@ -2378,15 +2378,21 @@
         <v>8</v>
       </c>
       <c r="BI45" t="s">
-        <v>26</v>
+        <v>8</v>
       </c>
       <c r="BJ45" t="s">
-        <v>26</v>
+        <v>8</v>
       </c>
       <c r="BK45" t="s">
-        <v>10</v>
-      </c>
-      <c r="BQ45" t="s">
+        <v>26</v>
+      </c>
+      <c r="BL45" t="s">
+        <v>26</v>
+      </c>
+      <c r="BM45" t="s">
+        <v>10</v>
+      </c>
+      <c r="BS45" t="s">
         <v>11</v>
       </c>
     </row>
@@ -2400,19 +2406,19 @@
       <c r="C46" t="s">
         <v>24</v>
       </c>
-      <c r="BB46" t="s">
-        <v>5</v>
-      </c>
-      <c r="BC46" t="s">
-        <v>6</v>
-      </c>
       <c r="BD46" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="BE46" t="s">
-        <v>10</v>
-      </c>
-      <c r="BR46" t="s">
+        <v>6</v>
+      </c>
+      <c r="BF46" t="s">
+        <v>8</v>
+      </c>
+      <c r="BG46" t="s">
+        <v>10</v>
+      </c>
+      <c r="BT46" t="s">
         <v>11</v>
       </c>
     </row>
@@ -2426,19 +2432,19 @@
       <c r="C47" t="s">
         <v>16</v>
       </c>
-      <c r="BC47" t="s">
-        <v>5</v>
-      </c>
-      <c r="BD47" t="s">
-        <v>6</v>
-      </c>
       <c r="BE47" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="BF47" t="s">
-        <v>10</v>
-      </c>
-      <c r="BS47" t="s">
+        <v>6</v>
+      </c>
+      <c r="BG47" t="s">
+        <v>8</v>
+      </c>
+      <c r="BH47" t="s">
+        <v>10</v>
+      </c>
+      <c r="BU47" t="s">
         <v>11</v>
       </c>
     </row>
@@ -2452,19 +2458,19 @@
       <c r="C48" t="s">
         <v>25</v>
       </c>
-      <c r="BD48" t="s">
-        <v>5</v>
-      </c>
-      <c r="BE48" t="s">
-        <v>6</v>
-      </c>
       <c r="BF48" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="BG48" t="s">
-        <v>10</v>
-      </c>
-      <c r="BT48" t="s">
+        <v>6</v>
+      </c>
+      <c r="BH48" t="s">
+        <v>8</v>
+      </c>
+      <c r="BI48" t="s">
+        <v>10</v>
+      </c>
+      <c r="BV48" t="s">
         <v>11</v>
       </c>
     </row>
@@ -2478,19 +2484,19 @@
       <c r="C49" t="s">
         <v>27</v>
       </c>
-      <c r="BE49" t="s">
-        <v>5</v>
-      </c>
-      <c r="BF49" t="s">
-        <v>6</v>
-      </c>
       <c r="BG49" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="BH49" t="s">
-        <v>10</v>
-      </c>
-      <c r="BU49" t="s">
+        <v>6</v>
+      </c>
+      <c r="BI49" t="s">
+        <v>8</v>
+      </c>
+      <c r="BJ49" t="s">
+        <v>10</v>
+      </c>
+      <c r="BW49" t="s">
         <v>11</v>
       </c>
     </row>
@@ -2504,23 +2510,17 @@
       <c r="C50" t="s">
         <v>28</v>
       </c>
-      <c r="BF50" t="s">
-        <v>5</v>
-      </c>
-      <c r="BG50" t="s">
-        <v>6</v>
-      </c>
       <c r="BH50" t="s">
+        <v>5</v>
+      </c>
+      <c r="BI50" t="s">
+        <v>6</v>
+      </c>
+      <c r="BJ50" t="s">
         <v>30</v>
       </c>
-      <c r="BI50" t="s">
+      <c r="BK50" t="s">
         <v>30</v>
-      </c>
-      <c r="BJ50" t="s">
-        <v>32</v>
-      </c>
-      <c r="BK50" t="s">
-        <v>32</v>
       </c>
       <c r="BL50" t="s">
         <v>32</v>
@@ -2532,10 +2532,10 @@
         <v>32</v>
       </c>
       <c r="BO50" t="s">
-        <v>8</v>
+        <v>32</v>
       </c>
       <c r="BP50" t="s">
-        <v>8</v>
+        <v>32</v>
       </c>
       <c r="BQ50" t="s">
         <v>8</v>
@@ -2544,9 +2544,15 @@
         <v>8</v>
       </c>
       <c r="BS50" t="s">
-        <v>10</v>
-      </c>
-      <c r="BV50" t="s">
+        <v>8</v>
+      </c>
+      <c r="BT50" t="s">
+        <v>8</v>
+      </c>
+      <c r="BU50" t="s">
+        <v>10</v>
+      </c>
+      <c r="BX50" t="s">
         <v>11</v>
       </c>
     </row>
@@ -2560,28 +2566,28 @@
       <c r="C51" t="s">
         <v>29</v>
       </c>
-      <c r="BG51" t="s">
-        <v>5</v>
-      </c>
-      <c r="BH51" t="s">
-        <v>6</v>
-      </c>
-      <c r="BK51" t="s">
+      <c r="BI51" t="s">
+        <v>5</v>
+      </c>
+      <c r="BJ51" t="s">
+        <v>6</v>
+      </c>
+      <c r="BM51" t="s">
         <v>21</v>
       </c>
-      <c r="BS51" t="s">
-        <v>8</v>
-      </c>
-      <c r="BT51" t="s">
-        <v>8</v>
-      </c>
       <c r="BU51" t="s">
         <v>8</v>
       </c>
       <c r="BV51" t="s">
-        <v>26</v>
+        <v>8</v>
       </c>
       <c r="BW51" t="s">
+        <v>8</v>
+      </c>
+      <c r="BX51" t="s">
+        <v>26</v>
+      </c>
+      <c r="BY51" t="s">
         <v>11</v>
       </c>
     </row>
@@ -2595,22 +2601,22 @@
       <c r="C52" t="s">
         <v>31</v>
       </c>
-      <c r="BH52" t="s">
-        <v>5</v>
-      </c>
-      <c r="BI52" t="s">
-        <v>6</v>
-      </c>
-      <c r="BL52" t="s">
+      <c r="BJ52" t="s">
+        <v>5</v>
+      </c>
+      <c r="BK52" t="s">
+        <v>6</v>
+      </c>
+      <c r="BN52" t="s">
         <v>21</v>
       </c>
-      <c r="BW52" t="s">
-        <v>8</v>
-      </c>
-      <c r="BX52" t="s">
-        <v>26</v>
-      </c>
       <c r="BY52" t="s">
+        <v>8</v>
+      </c>
+      <c r="BZ52" t="s">
+        <v>26</v>
+      </c>
+      <c r="CA52" t="s">
         <v>11</v>
       </c>
     </row>
@@ -2624,19 +2630,19 @@
       <c r="C53" t="s">
         <v>33</v>
       </c>
-      <c r="BI53" t="s">
-        <v>5</v>
-      </c>
-      <c r="BJ53" t="s">
-        <v>6</v>
-      </c>
-      <c r="BM53" t="s">
-        <v>8</v>
-      </c>
-      <c r="BN53" t="s">
-        <v>10</v>
-      </c>
-      <c r="BZ53" t="s">
+      <c r="BK53" t="s">
+        <v>5</v>
+      </c>
+      <c r="BL53" t="s">
+        <v>6</v>
+      </c>
+      <c r="BO53" t="s">
+        <v>8</v>
+      </c>
+      <c r="BP53" t="s">
+        <v>10</v>
+      </c>
+      <c r="CB53" t="s">
         <v>11</v>
       </c>
     </row>
@@ -2650,19 +2656,19 @@
       <c r="C54" t="s">
         <v>34</v>
       </c>
-      <c r="BJ54" t="s">
-        <v>5</v>
-      </c>
-      <c r="BK54" t="s">
-        <v>6</v>
-      </c>
-      <c r="BN54" t="s">
-        <v>8</v>
-      </c>
-      <c r="BO54" t="s">
-        <v>10</v>
-      </c>
-      <c r="CA54" t="s">
+      <c r="BL54" t="s">
+        <v>5</v>
+      </c>
+      <c r="BM54" t="s">
+        <v>6</v>
+      </c>
+      <c r="BP54" t="s">
+        <v>8</v>
+      </c>
+      <c r="BQ54" t="s">
+        <v>10</v>
+      </c>
+      <c r="CC54" t="s">
         <v>11</v>
       </c>
     </row>
@@ -2676,19 +2682,19 @@
       <c r="C55" t="s">
         <v>27</v>
       </c>
-      <c r="BK55" t="s">
-        <v>5</v>
-      </c>
-      <c r="BL55" t="s">
-        <v>6</v>
-      </c>
-      <c r="BO55" t="s">
-        <v>8</v>
-      </c>
-      <c r="BP55" t="s">
-        <v>10</v>
-      </c>
-      <c r="CB55" t="s">
+      <c r="BM55" t="s">
+        <v>5</v>
+      </c>
+      <c r="BN55" t="s">
+        <v>6</v>
+      </c>
+      <c r="BQ55" t="s">
+        <v>8</v>
+      </c>
+      <c r="BR55" t="s">
+        <v>10</v>
+      </c>
+      <c r="CD55" t="s">
         <v>11</v>
       </c>
     </row>
@@ -2702,26 +2708,20 @@
       <c r="C56" t="s">
         <v>28</v>
       </c>
-      <c r="BL56" t="s">
-        <v>5</v>
-      </c>
-      <c r="BM56" t="s">
-        <v>6</v>
-      </c>
-      <c r="BP56" t="s">
-        <v>32</v>
-      </c>
-      <c r="BQ56" t="s">
-        <v>32</v>
+      <c r="BN56" t="s">
+        <v>5</v>
+      </c>
+      <c r="BO56" t="s">
+        <v>6</v>
       </c>
       <c r="BR56" t="s">
         <v>32</v>
       </c>
       <c r="BS56" t="s">
-        <v>8</v>
+        <v>32</v>
       </c>
       <c r="BT56" t="s">
-        <v>8</v>
+        <v>32</v>
       </c>
       <c r="BU56" t="s">
         <v>8</v>
@@ -2730,12 +2730,18 @@
         <v>8</v>
       </c>
       <c r="BW56" t="s">
-        <v>26</v>
+        <v>8</v>
       </c>
       <c r="BX56" t="s">
-        <v>10</v>
-      </c>
-      <c r="CC56" t="s">
+        <v>8</v>
+      </c>
+      <c r="BY56" t="s">
+        <v>26</v>
+      </c>
+      <c r="BZ56" t="s">
+        <v>10</v>
+      </c>
+      <c r="CE56" t="s">
         <v>11</v>
       </c>
     </row>
@@ -2749,31 +2755,31 @@
       <c r="C57" t="s">
         <v>29</v>
       </c>
-      <c r="BM57" t="s">
-        <v>5</v>
-      </c>
-      <c r="BN57" t="s">
-        <v>6</v>
-      </c>
-      <c r="BQ57" t="s">
+      <c r="BO57" t="s">
+        <v>5</v>
+      </c>
+      <c r="BP57" t="s">
+        <v>6</v>
+      </c>
+      <c r="BS57" t="s">
         <v>21</v>
       </c>
-      <c r="BX57" t="s">
-        <v>8</v>
-      </c>
-      <c r="BY57" t="s">
-        <v>8</v>
-      </c>
       <c r="BZ57" t="s">
         <v>8</v>
       </c>
       <c r="CA57" t="s">
-        <v>26</v>
+        <v>8</v>
       </c>
       <c r="CB57" t="s">
-        <v>10</v>
+        <v>8</v>
+      </c>
+      <c r="CC57" t="s">
+        <v>26</v>
       </c>
       <c r="CD57" t="s">
+        <v>10</v>
+      </c>
+      <c r="CF57" t="s">
         <v>11</v>
       </c>
     </row>
@@ -2787,25 +2793,25 @@
       <c r="C58" t="s">
         <v>31</v>
       </c>
-      <c r="BN58" t="s">
-        <v>5</v>
-      </c>
-      <c r="BO58" t="s">
-        <v>6</v>
-      </c>
-      <c r="BR58" t="s">
+      <c r="BP58" t="s">
+        <v>5</v>
+      </c>
+      <c r="BQ58" t="s">
+        <v>6</v>
+      </c>
+      <c r="BT58" t="s">
         <v>21</v>
       </c>
-      <c r="CB58" t="s">
-        <v>8</v>
-      </c>
-      <c r="CC58" t="s">
-        <v>26</v>
-      </c>
       <c r="CD58" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="CE58" t="s">
+        <v>26</v>
+      </c>
+      <c r="CF58" t="s">
+        <v>10</v>
+      </c>
+      <c r="CG58" t="s">
         <v>11</v>
       </c>
     </row>
@@ -2819,19 +2825,19 @@
       <c r="C59" t="s">
         <v>33</v>
       </c>
-      <c r="BO59" t="s">
-        <v>5</v>
-      </c>
-      <c r="BP59" t="s">
-        <v>6</v>
-      </c>
-      <c r="BS59" t="s">
-        <v>8</v>
-      </c>
-      <c r="BT59" t="s">
-        <v>10</v>
-      </c>
-      <c r="CF59" t="s">
+      <c r="BQ59" t="s">
+        <v>5</v>
+      </c>
+      <c r="BR59" t="s">
+        <v>6</v>
+      </c>
+      <c r="BU59" t="s">
+        <v>8</v>
+      </c>
+      <c r="BV59" t="s">
+        <v>10</v>
+      </c>
+      <c r="CH59" t="s">
         <v>11</v>
       </c>
     </row>
@@ -2845,19 +2851,19 @@
       <c r="C60" t="s">
         <v>34</v>
       </c>
-      <c r="BP60" t="s">
-        <v>5</v>
-      </c>
-      <c r="BQ60" t="s">
-        <v>6</v>
-      </c>
-      <c r="BT60" t="s">
-        <v>8</v>
-      </c>
-      <c r="BU60" t="s">
-        <v>10</v>
-      </c>
-      <c r="CG60" t="s">
+      <c r="BR60" t="s">
+        <v>5</v>
+      </c>
+      <c r="BS60" t="s">
+        <v>6</v>
+      </c>
+      <c r="BV60" t="s">
+        <v>8</v>
+      </c>
+      <c r="BW60" t="s">
+        <v>10</v>
+      </c>
+      <c r="CI60" t="s">
         <v>11</v>
       </c>
     </row>
@@ -2871,19 +2877,19 @@
       <c r="C61" t="s">
         <v>27</v>
       </c>
-      <c r="BQ61" t="s">
-        <v>5</v>
-      </c>
-      <c r="BR61" t="s">
-        <v>6</v>
-      </c>
-      <c r="BU61" t="s">
-        <v>8</v>
-      </c>
-      <c r="BV61" t="s">
-        <v>10</v>
-      </c>
-      <c r="CH61" t="s">
+      <c r="BS61" t="s">
+        <v>5</v>
+      </c>
+      <c r="BT61" t="s">
+        <v>6</v>
+      </c>
+      <c r="BW61" t="s">
+        <v>8</v>
+      </c>
+      <c r="BX61" t="s">
+        <v>10</v>
+      </c>
+      <c r="CJ61" t="s">
         <v>11</v>
       </c>
     </row>
@@ -2897,24 +2903,18 @@
       <c r="C62" t="s">
         <v>28</v>
       </c>
-      <c r="BR62" t="s">
-        <v>5</v>
-      </c>
-      <c r="BS62" t="s">
-        <v>6</v>
-      </c>
-      <c r="BV62" t="s">
+      <c r="BT62" t="s">
+        <v>5</v>
+      </c>
+      <c r="BU62" t="s">
+        <v>6</v>
+      </c>
+      <c r="BX62" t="s">
         <v>32</v>
       </c>
-      <c r="BW62" t="s">
+      <c r="BY62" t="s">
         <v>32</v>
       </c>
-      <c r="BX62" t="s">
-        <v>8</v>
-      </c>
-      <c r="BY62" t="s">
-        <v>8</v>
-      </c>
       <c r="BZ62" t="s">
         <v>8</v>
       </c>
@@ -2922,12 +2922,18 @@
         <v>8</v>
       </c>
       <c r="CB62" t="s">
-        <v>26</v>
+        <v>8</v>
       </c>
       <c r="CC62" t="s">
-        <v>10</v>
-      </c>
-      <c r="CI62" t="s">
+        <v>8</v>
+      </c>
+      <c r="CD62" t="s">
+        <v>26</v>
+      </c>
+      <c r="CE62" t="s">
+        <v>10</v>
+      </c>
+      <c r="CK62" t="s">
         <v>11</v>
       </c>
     </row>
@@ -2941,28 +2947,28 @@
       <c r="C63" t="s">
         <v>29</v>
       </c>
-      <c r="BS63" t="s">
-        <v>5</v>
-      </c>
-      <c r="BT63" t="s">
-        <v>6</v>
-      </c>
-      <c r="BW63" t="s">
+      <c r="BU63" t="s">
+        <v>5</v>
+      </c>
+      <c r="BV63" t="s">
+        <v>6</v>
+      </c>
+      <c r="BY63" t="s">
         <v>21</v>
       </c>
-      <c r="CC63" t="s">
-        <v>8</v>
-      </c>
-      <c r="CD63" t="s">
-        <v>8</v>
-      </c>
       <c r="CE63" t="s">
         <v>8</v>
       </c>
       <c r="CF63" t="s">
-        <v>10</v>
-      </c>
-      <c r="CJ63" t="s">
+        <v>8</v>
+      </c>
+      <c r="CG63" t="s">
+        <v>8</v>
+      </c>
+      <c r="CH63" t="s">
+        <v>10</v>
+      </c>
+      <c r="CL63" t="s">
         <v>11</v>
       </c>
     </row>
@@ -2976,31 +2982,31 @@
       <c r="C64" t="s">
         <v>31</v>
       </c>
-      <c r="BT64" t="s">
-        <v>5</v>
-      </c>
-      <c r="BU64" t="s">
-        <v>6</v>
-      </c>
-      <c r="BX64" t="s">
+      <c r="BV64" t="s">
+        <v>5</v>
+      </c>
+      <c r="BW64" t="s">
+        <v>6</v>
+      </c>
+      <c r="BZ64" t="s">
         <v>30</v>
       </c>
-      <c r="BY64" t="s">
+      <c r="CA64" t="s">
         <v>21</v>
       </c>
-      <c r="CF64" t="s">
-        <v>8</v>
-      </c>
-      <c r="CG64" t="s">
-        <v>26</v>
-      </c>
       <c r="CH64" t="s">
-        <v>26</v>
+        <v>8</v>
       </c>
       <c r="CI64" t="s">
-        <v>10</v>
+        <v>26</v>
+      </c>
+      <c r="CJ64" t="s">
+        <v>26</v>
       </c>
       <c r="CK64" t="s">
+        <v>10</v>
+      </c>
+      <c r="CM64" t="s">
         <v>11</v>
       </c>
     </row>
@@ -3014,19 +3020,19 @@
       <c r="C65" t="s">
         <v>33</v>
       </c>
-      <c r="BU65" t="s">
-        <v>5</v>
-      </c>
-      <c r="BV65" t="s">
-        <v>6</v>
-      </c>
-      <c r="BZ65" t="s">
-        <v>8</v>
-      </c>
-      <c r="CA65" t="s">
-        <v>10</v>
-      </c>
-      <c r="CL65" t="s">
+      <c r="BW65" t="s">
+        <v>5</v>
+      </c>
+      <c r="BX65" t="s">
+        <v>6</v>
+      </c>
+      <c r="CB65" t="s">
+        <v>8</v>
+      </c>
+      <c r="CC65" t="s">
+        <v>10</v>
+      </c>
+      <c r="CN65" t="s">
         <v>11</v>
       </c>
     </row>
@@ -3040,19 +3046,19 @@
       <c r="C66" t="s">
         <v>34</v>
       </c>
-      <c r="BV66" t="s">
-        <v>5</v>
-      </c>
-      <c r="BW66" t="s">
-        <v>6</v>
-      </c>
-      <c r="CA66" t="s">
-        <v>8</v>
-      </c>
-      <c r="CB66" t="s">
-        <v>10</v>
-      </c>
-      <c r="CM66" t="s">
+      <c r="BX66" t="s">
+        <v>5</v>
+      </c>
+      <c r="BY66" t="s">
+        <v>6</v>
+      </c>
+      <c r="CC66" t="s">
+        <v>8</v>
+      </c>
+      <c r="CD66" t="s">
+        <v>10</v>
+      </c>
+      <c r="CO66" t="s">
         <v>11</v>
       </c>
     </row>
@@ -3066,28 +3072,28 @@
       <c r="C67" t="s">
         <v>35</v>
       </c>
-      <c r="CB67" t="s">
-        <v>5</v>
-      </c>
-      <c r="CC67" t="s">
-        <v>6</v>
-      </c>
       <c r="CD67" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="CE67" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="CF67" t="s">
         <v>8</v>
       </c>
       <c r="CG67" t="s">
-        <v>26</v>
+        <v>8</v>
       </c>
       <c r="CH67" t="s">
-        <v>10</v>
-      </c>
-      <c r="CN67" t="s">
+        <v>8</v>
+      </c>
+      <c r="CI67" t="s">
+        <v>26</v>
+      </c>
+      <c r="CJ67" t="s">
+        <v>10</v>
+      </c>
+      <c r="CP67" t="s">
         <v>11</v>
       </c>
     </row>
@@ -3101,28 +3107,28 @@
       <c r="C68" t="s">
         <v>36</v>
       </c>
-      <c r="CC68" t="s">
-        <v>5</v>
-      </c>
-      <c r="CD68" t="s">
-        <v>6</v>
-      </c>
       <c r="CE68" t="s">
+        <v>5</v>
+      </c>
+      <c r="CF68" t="s">
+        <v>6</v>
+      </c>
+      <c r="CG68" t="s">
         <v>21</v>
       </c>
-      <c r="CH68" t="s">
-        <v>8</v>
-      </c>
-      <c r="CI68" t="s">
-        <v>8</v>
-      </c>
       <c r="CJ68" t="s">
         <v>8</v>
       </c>
       <c r="CK68" t="s">
-        <v>10</v>
-      </c>
-      <c r="CO68" t="s">
+        <v>8</v>
+      </c>
+      <c r="CL68" t="s">
+        <v>8</v>
+      </c>
+      <c r="CM68" t="s">
+        <v>10</v>
+      </c>
+      <c r="CQ68" t="s">
         <v>11</v>
       </c>
     </row>
@@ -3136,19 +3142,19 @@
       <c r="C69" t="s">
         <v>37</v>
       </c>
-      <c r="CD69" t="s">
-        <v>5</v>
-      </c>
-      <c r="CE69" t="s">
-        <v>6</v>
-      </c>
       <c r="CF69" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="CG69" t="s">
-        <v>10</v>
-      </c>
-      <c r="CP69" t="s">
+        <v>6</v>
+      </c>
+      <c r="CH69" t="s">
+        <v>8</v>
+      </c>
+      <c r="CI69" t="s">
+        <v>10</v>
+      </c>
+      <c r="CR69" t="s">
         <v>11</v>
       </c>
     </row>
@@ -3162,19 +3168,19 @@
       <c r="C70" t="s">
         <v>38</v>
       </c>
-      <c r="CE70" t="s">
-        <v>5</v>
-      </c>
-      <c r="CF70" t="s">
-        <v>6</v>
-      </c>
       <c r="CG70" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="CH70" t="s">
-        <v>10</v>
-      </c>
-      <c r="CQ70" t="s">
+        <v>6</v>
+      </c>
+      <c r="CI70" t="s">
+        <v>8</v>
+      </c>
+      <c r="CJ70" t="s">
+        <v>10</v>
+      </c>
+      <c r="CS70" t="s">
         <v>11</v>
       </c>
     </row>
@@ -3188,28 +3194,28 @@
       <c r="C71" t="s">
         <v>18</v>
       </c>
-      <c r="CF71" t="s">
-        <v>5</v>
-      </c>
-      <c r="CG71" t="s">
-        <v>6</v>
-      </c>
       <c r="CH71" t="s">
+        <v>5</v>
+      </c>
+      <c r="CI71" t="s">
+        <v>6</v>
+      </c>
+      <c r="CJ71" t="s">
         <v>32</v>
       </c>
-      <c r="CI71" t="s">
-        <v>8</v>
-      </c>
-      <c r="CJ71" t="s">
-        <v>8</v>
-      </c>
       <c r="CK71" t="s">
         <v>8</v>
       </c>
       <c r="CL71" t="s">
-        <v>10</v>
-      </c>
-      <c r="CR71" t="s">
+        <v>8</v>
+      </c>
+      <c r="CM71" t="s">
+        <v>8</v>
+      </c>
+      <c r="CN71" t="s">
+        <v>10</v>
+      </c>
+      <c r="CT71" t="s">
         <v>11</v>
       </c>
     </row>
@@ -3223,37 +3229,37 @@
       <c r="C72" t="s">
         <v>19</v>
       </c>
-      <c r="CG72" t="s">
-        <v>5</v>
-      </c>
-      <c r="CH72" t="s">
-        <v>6</v>
-      </c>
       <c r="CI72" t="s">
+        <v>5</v>
+      </c>
+      <c r="CJ72" t="s">
+        <v>6</v>
+      </c>
+      <c r="CK72" t="s">
         <v>21</v>
       </c>
-      <c r="CL72" t="s">
-        <v>8</v>
-      </c>
-      <c r="CM72" t="s">
-        <v>8</v>
-      </c>
       <c r="CN72" t="s">
         <v>8</v>
       </c>
       <c r="CO72" t="s">
-        <v>26</v>
+        <v>8</v>
       </c>
       <c r="CP72" t="s">
-        <v>26</v>
+        <v>8</v>
       </c>
       <c r="CQ72" t="s">
         <v>26</v>
       </c>
       <c r="CR72" t="s">
-        <v>10</v>
+        <v>26</v>
       </c>
       <c r="CS72" t="s">
+        <v>26</v>
+      </c>
+      <c r="CT72" t="s">
+        <v>10</v>
+      </c>
+      <c r="CU72" t="s">
         <v>11</v>
       </c>
     </row>
@@ -3267,24 +3273,18 @@
       <c r="C73" t="s">
         <v>20</v>
       </c>
-      <c r="CH73" t="s">
-        <v>5</v>
-      </c>
-      <c r="CI73" t="s">
-        <v>6</v>
-      </c>
       <c r="CJ73" t="s">
+        <v>5</v>
+      </c>
+      <c r="CK73" t="s">
+        <v>6</v>
+      </c>
+      <c r="CL73" t="s">
         <v>21</v>
       </c>
-      <c r="CR73" t="s">
+      <c r="CT73" t="s">
         <v>32</v>
       </c>
-      <c r="CS73" t="s">
-        <v>8</v>
-      </c>
-      <c r="CT73" t="s">
-        <v>8</v>
-      </c>
       <c r="CU73" t="s">
         <v>8</v>
       </c>
@@ -3292,9 +3292,15 @@
         <v>8</v>
       </c>
       <c r="CW73" t="s">
-        <v>26</v>
+        <v>8</v>
       </c>
       <c r="CX73" t="s">
+        <v>8</v>
+      </c>
+      <c r="CY73" t="s">
+        <v>26</v>
+      </c>
+      <c r="CZ73" t="s">
         <v>11</v>
       </c>
     </row>
@@ -3308,17 +3314,11 @@
       <c r="C74" t="s">
         <v>22</v>
       </c>
-      <c r="CI74" t="s">
-        <v>5</v>
-      </c>
-      <c r="CJ74" t="s">
-        <v>6</v>
-      </c>
       <c r="CK74" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="CL74" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="CM74" t="s">
         <v>8</v>
@@ -3327,10 +3327,10 @@
         <v>8</v>
       </c>
       <c r="CO74" t="s">
-        <v>26</v>
+        <v>8</v>
       </c>
       <c r="CP74" t="s">
-        <v>26</v>
+        <v>8</v>
       </c>
       <c r="CQ74" t="s">
         <v>26</v>
@@ -3339,9 +3339,15 @@
         <v>26</v>
       </c>
       <c r="CS74" t="s">
-        <v>10</v>
-      </c>
-      <c r="CY74" t="s">
+        <v>26</v>
+      </c>
+      <c r="CT74" t="s">
+        <v>26</v>
+      </c>
+      <c r="CU74" t="s">
+        <v>10</v>
+      </c>
+      <c r="DA74" t="s">
         <v>11</v>
       </c>
     </row>
@@ -3355,17 +3361,11 @@
       <c r="C75" t="s">
         <v>23</v>
       </c>
-      <c r="CJ75" t="s">
-        <v>5</v>
-      </c>
-      <c r="CK75" t="s">
-        <v>6</v>
-      </c>
       <c r="CL75" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="CM75" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="CN75" t="s">
         <v>8</v>
@@ -3380,15 +3380,21 @@
         <v>8</v>
       </c>
       <c r="CR75" t="s">
-        <v>26</v>
+        <v>8</v>
       </c>
       <c r="CS75" t="s">
-        <v>26</v>
+        <v>8</v>
       </c>
       <c r="CT75" t="s">
-        <v>10</v>
-      </c>
-      <c r="CZ75" t="s">
+        <v>26</v>
+      </c>
+      <c r="CU75" t="s">
+        <v>26</v>
+      </c>
+      <c r="CV75" t="s">
+        <v>10</v>
+      </c>
+      <c r="DB75" t="s">
         <v>11</v>
       </c>
     </row>
@@ -3402,19 +3408,19 @@
       <c r="C76" t="s">
         <v>24</v>
       </c>
-      <c r="CK76" t="s">
-        <v>5</v>
-      </c>
-      <c r="CL76" t="s">
-        <v>6</v>
-      </c>
       <c r="CM76" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="CN76" t="s">
-        <v>10</v>
-      </c>
-      <c r="DA76" t="s">
+        <v>6</v>
+      </c>
+      <c r="CO76" t="s">
+        <v>8</v>
+      </c>
+      <c r="CP76" t="s">
+        <v>10</v>
+      </c>
+      <c r="DC76" t="s">
         <v>11</v>
       </c>
     </row>
@@ -3428,19 +3434,19 @@
       <c r="C77" t="s">
         <v>16</v>
       </c>
-      <c r="CL77" t="s">
-        <v>5</v>
-      </c>
-      <c r="CM77" t="s">
-        <v>6</v>
-      </c>
       <c r="CN77" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="CO77" t="s">
-        <v>10</v>
-      </c>
-      <c r="DB77" t="s">
+        <v>6</v>
+      </c>
+      <c r="CP77" t="s">
+        <v>8</v>
+      </c>
+      <c r="CQ77" t="s">
+        <v>10</v>
+      </c>
+      <c r="DD77" t="s">
         <v>11</v>
       </c>
     </row>
@@ -3454,19 +3460,19 @@
       <c r="C78" t="s">
         <v>25</v>
       </c>
-      <c r="CM78" t="s">
-        <v>5</v>
-      </c>
-      <c r="CN78" t="s">
-        <v>6</v>
-      </c>
       <c r="CO78" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="CP78" t="s">
-        <v>10</v>
-      </c>
-      <c r="DC78" t="s">
+        <v>6</v>
+      </c>
+      <c r="CQ78" t="s">
+        <v>8</v>
+      </c>
+      <c r="CR78" t="s">
+        <v>10</v>
+      </c>
+      <c r="DE78" t="s">
         <v>11</v>
       </c>
     </row>
@@ -3480,19 +3486,19 @@
       <c r="C79" t="s">
         <v>27</v>
       </c>
-      <c r="CN79" t="s">
-        <v>5</v>
-      </c>
-      <c r="CO79" t="s">
-        <v>6</v>
-      </c>
       <c r="CP79" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="CQ79" t="s">
-        <v>10</v>
-      </c>
-      <c r="DD79" t="s">
+        <v>6</v>
+      </c>
+      <c r="CR79" t="s">
+        <v>8</v>
+      </c>
+      <c r="CS79" t="s">
+        <v>10</v>
+      </c>
+      <c r="DF79" t="s">
         <v>11</v>
       </c>
     </row>
@@ -3506,23 +3512,17 @@
       <c r="C80" t="s">
         <v>28</v>
       </c>
-      <c r="CO80" t="s">
-        <v>5</v>
-      </c>
-      <c r="CP80" t="s">
-        <v>6</v>
-      </c>
       <c r="CQ80" t="s">
+        <v>5</v>
+      </c>
+      <c r="CR80" t="s">
+        <v>6</v>
+      </c>
+      <c r="CS80" t="s">
         <v>30</v>
       </c>
-      <c r="CR80" t="s">
+      <c r="CT80" t="s">
         <v>30</v>
-      </c>
-      <c r="CS80" t="s">
-        <v>32</v>
-      </c>
-      <c r="CT80" t="s">
-        <v>32</v>
       </c>
       <c r="CU80" t="s">
         <v>32</v>
@@ -3534,10 +3534,10 @@
         <v>32</v>
       </c>
       <c r="CX80" t="s">
-        <v>8</v>
+        <v>32</v>
       </c>
       <c r="CY80" t="s">
-        <v>8</v>
+        <v>32</v>
       </c>
       <c r="CZ80" t="s">
         <v>8</v>
@@ -3546,9 +3546,15 @@
         <v>8</v>
       </c>
       <c r="DB80" t="s">
-        <v>10</v>
-      </c>
-      <c r="DE80" t="s">
+        <v>8</v>
+      </c>
+      <c r="DC80" t="s">
+        <v>8</v>
+      </c>
+      <c r="DD80" t="s">
+        <v>10</v>
+      </c>
+      <c r="DG80" t="s">
         <v>11</v>
       </c>
     </row>
@@ -3562,28 +3568,28 @@
       <c r="C81" t="s">
         <v>29</v>
       </c>
-      <c r="CP81" t="s">
-        <v>5</v>
-      </c>
-      <c r="CQ81" t="s">
-        <v>6</v>
-      </c>
-      <c r="CT81" t="s">
+      <c r="CR81" t="s">
+        <v>5</v>
+      </c>
+      <c r="CS81" t="s">
+        <v>6</v>
+      </c>
+      <c r="CV81" t="s">
         <v>21</v>
       </c>
-      <c r="DB81" t="s">
-        <v>8</v>
-      </c>
-      <c r="DC81" t="s">
-        <v>8</v>
-      </c>
       <c r="DD81" t="s">
         <v>8</v>
       </c>
       <c r="DE81" t="s">
-        <v>26</v>
+        <v>8</v>
       </c>
       <c r="DF81" t="s">
+        <v>8</v>
+      </c>
+      <c r="DG81" t="s">
+        <v>26</v>
+      </c>
+      <c r="DH81" t="s">
         <v>11</v>
       </c>
     </row>
@@ -3597,22 +3603,22 @@
       <c r="C82" t="s">
         <v>31</v>
       </c>
-      <c r="CQ82" t="s">
-        <v>5</v>
-      </c>
-      <c r="CR82" t="s">
-        <v>6</v>
-      </c>
-      <c r="CU82" t="s">
+      <c r="CS82" t="s">
+        <v>5</v>
+      </c>
+      <c r="CT82" t="s">
+        <v>6</v>
+      </c>
+      <c r="CW82" t="s">
         <v>21</v>
       </c>
-      <c r="DF82" t="s">
-        <v>8</v>
-      </c>
-      <c r="DG82" t="s">
-        <v>26</v>
-      </c>
       <c r="DH82" t="s">
+        <v>8</v>
+      </c>
+      <c r="DI82" t="s">
+        <v>26</v>
+      </c>
+      <c r="DJ82" t="s">
         <v>11</v>
       </c>
     </row>
@@ -3626,19 +3632,19 @@
       <c r="C83" t="s">
         <v>33</v>
       </c>
-      <c r="CR83" t="s">
-        <v>5</v>
-      </c>
-      <c r="CS83" t="s">
-        <v>6</v>
-      </c>
-      <c r="CV83" t="s">
-        <v>8</v>
-      </c>
-      <c r="CW83" t="s">
-        <v>10</v>
-      </c>
-      <c r="DI83" t="s">
+      <c r="CT83" t="s">
+        <v>5</v>
+      </c>
+      <c r="CU83" t="s">
+        <v>6</v>
+      </c>
+      <c r="CX83" t="s">
+        <v>8</v>
+      </c>
+      <c r="CY83" t="s">
+        <v>10</v>
+      </c>
+      <c r="DK83" t="s">
         <v>11</v>
       </c>
     </row>
@@ -3652,19 +3658,19 @@
       <c r="C84" t="s">
         <v>34</v>
       </c>
-      <c r="CS84" t="s">
-        <v>5</v>
-      </c>
-      <c r="CT84" t="s">
-        <v>6</v>
-      </c>
-      <c r="CW84" t="s">
-        <v>8</v>
-      </c>
-      <c r="CX84" t="s">
-        <v>10</v>
-      </c>
-      <c r="DJ84" t="s">
+      <c r="CU84" t="s">
+        <v>5</v>
+      </c>
+      <c r="CV84" t="s">
+        <v>6</v>
+      </c>
+      <c r="CY84" t="s">
+        <v>8</v>
+      </c>
+      <c r="CZ84" t="s">
+        <v>10</v>
+      </c>
+      <c r="DL84" t="s">
         <v>11</v>
       </c>
     </row>
@@ -3678,19 +3684,19 @@
       <c r="C85" t="s">
         <v>27</v>
       </c>
-      <c r="CT85" t="s">
-        <v>5</v>
-      </c>
-      <c r="CU85" t="s">
-        <v>6</v>
-      </c>
-      <c r="CX85" t="s">
-        <v>8</v>
-      </c>
-      <c r="CY85" t="s">
-        <v>10</v>
-      </c>
-      <c r="DK85" t="s">
+      <c r="CV85" t="s">
+        <v>5</v>
+      </c>
+      <c r="CW85" t="s">
+        <v>6</v>
+      </c>
+      <c r="CZ85" t="s">
+        <v>8</v>
+      </c>
+      <c r="DA85" t="s">
+        <v>10</v>
+      </c>
+      <c r="DM85" t="s">
         <v>11</v>
       </c>
     </row>
@@ -3704,26 +3710,20 @@
       <c r="C86" t="s">
         <v>28</v>
       </c>
-      <c r="CU86" t="s">
-        <v>5</v>
-      </c>
-      <c r="CV86" t="s">
-        <v>6</v>
-      </c>
-      <c r="CY86" t="s">
-        <v>32</v>
-      </c>
-      <c r="CZ86" t="s">
-        <v>32</v>
+      <c r="CW86" t="s">
+        <v>5</v>
+      </c>
+      <c r="CX86" t="s">
+        <v>6</v>
       </c>
       <c r="DA86" t="s">
         <v>32</v>
       </c>
       <c r="DB86" t="s">
-        <v>8</v>
+        <v>32</v>
       </c>
       <c r="DC86" t="s">
-        <v>8</v>
+        <v>32</v>
       </c>
       <c r="DD86" t="s">
         <v>8</v>
@@ -3732,12 +3732,18 @@
         <v>8</v>
       </c>
       <c r="DF86" t="s">
-        <v>26</v>
+        <v>8</v>
       </c>
       <c r="DG86" t="s">
-        <v>10</v>
-      </c>
-      <c r="DL86" t="s">
+        <v>8</v>
+      </c>
+      <c r="DH86" t="s">
+        <v>26</v>
+      </c>
+      <c r="DI86" t="s">
+        <v>10</v>
+      </c>
+      <c r="DN86" t="s">
         <v>11</v>
       </c>
     </row>
@@ -3751,31 +3757,31 @@
       <c r="C87" t="s">
         <v>29</v>
       </c>
-      <c r="CV87" t="s">
-        <v>5</v>
-      </c>
-      <c r="CW87" t="s">
-        <v>6</v>
-      </c>
-      <c r="CZ87" t="s">
+      <c r="CX87" t="s">
+        <v>5</v>
+      </c>
+      <c r="CY87" t="s">
+        <v>6</v>
+      </c>
+      <c r="DB87" t="s">
         <v>21</v>
       </c>
-      <c r="DG87" t="s">
-        <v>8</v>
-      </c>
-      <c r="DH87" t="s">
-        <v>8</v>
-      </c>
       <c r="DI87" t="s">
         <v>8</v>
       </c>
       <c r="DJ87" t="s">
-        <v>26</v>
+        <v>8</v>
       </c>
       <c r="DK87" t="s">
-        <v>10</v>
+        <v>8</v>
+      </c>
+      <c r="DL87" t="s">
+        <v>26</v>
       </c>
       <c r="DM87" t="s">
+        <v>10</v>
+      </c>
+      <c r="DO87" t="s">
         <v>11</v>
       </c>
     </row>
@@ -3789,25 +3795,25 @@
       <c r="C88" t="s">
         <v>31</v>
       </c>
-      <c r="CW88" t="s">
-        <v>5</v>
-      </c>
-      <c r="CX88" t="s">
-        <v>6</v>
-      </c>
-      <c r="DA88" t="s">
+      <c r="CY88" t="s">
+        <v>5</v>
+      </c>
+      <c r="CZ88" t="s">
+        <v>6</v>
+      </c>
+      <c r="DC88" t="s">
         <v>21</v>
       </c>
-      <c r="DK88" t="s">
-        <v>8</v>
-      </c>
-      <c r="DL88" t="s">
-        <v>26</v>
-      </c>
       <c r="DM88" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="DN88" t="s">
+        <v>26</v>
+      </c>
+      <c r="DO88" t="s">
+        <v>10</v>
+      </c>
+      <c r="DP88" t="s">
         <v>11</v>
       </c>
     </row>
@@ -3821,19 +3827,19 @@
       <c r="C89" t="s">
         <v>33</v>
       </c>
-      <c r="CX89" t="s">
-        <v>5</v>
-      </c>
-      <c r="CY89" t="s">
-        <v>6</v>
-      </c>
-      <c r="DB89" t="s">
-        <v>8</v>
-      </c>
-      <c r="DC89" t="s">
-        <v>10</v>
-      </c>
-      <c r="DO89" t="s">
+      <c r="CZ89" t="s">
+        <v>5</v>
+      </c>
+      <c r="DA89" t="s">
+        <v>6</v>
+      </c>
+      <c r="DD89" t="s">
+        <v>8</v>
+      </c>
+      <c r="DE89" t="s">
+        <v>10</v>
+      </c>
+      <c r="DQ89" t="s">
         <v>11</v>
       </c>
     </row>
@@ -3847,19 +3853,19 @@
       <c r="C90" t="s">
         <v>34</v>
       </c>
-      <c r="CY90" t="s">
-        <v>5</v>
-      </c>
-      <c r="CZ90" t="s">
-        <v>6</v>
-      </c>
-      <c r="DC90" t="s">
-        <v>8</v>
-      </c>
-      <c r="DD90" t="s">
-        <v>10</v>
-      </c>
-      <c r="DP90" t="s">
+      <c r="DA90" t="s">
+        <v>5</v>
+      </c>
+      <c r="DB90" t="s">
+        <v>6</v>
+      </c>
+      <c r="DE90" t="s">
+        <v>8</v>
+      </c>
+      <c r="DF90" t="s">
+        <v>10</v>
+      </c>
+      <c r="DR90" t="s">
         <v>11</v>
       </c>
     </row>
@@ -3873,19 +3879,19 @@
       <c r="C91" t="s">
         <v>27</v>
       </c>
-      <c r="CZ91" t="s">
-        <v>5</v>
-      </c>
-      <c r="DA91" t="s">
-        <v>6</v>
-      </c>
-      <c r="DD91" t="s">
-        <v>8</v>
-      </c>
-      <c r="DE91" t="s">
-        <v>10</v>
-      </c>
-      <c r="DQ91" t="s">
+      <c r="DB91" t="s">
+        <v>5</v>
+      </c>
+      <c r="DC91" t="s">
+        <v>6</v>
+      </c>
+      <c r="DF91" t="s">
+        <v>8</v>
+      </c>
+      <c r="DG91" t="s">
+        <v>10</v>
+      </c>
+      <c r="DS91" t="s">
         <v>11</v>
       </c>
     </row>
@@ -3899,24 +3905,18 @@
       <c r="C92" t="s">
         <v>28</v>
       </c>
-      <c r="DA92" t="s">
-        <v>5</v>
-      </c>
-      <c r="DB92" t="s">
-        <v>6</v>
-      </c>
-      <c r="DE92" t="s">
+      <c r="DC92" t="s">
+        <v>5</v>
+      </c>
+      <c r="DD92" t="s">
+        <v>6</v>
+      </c>
+      <c r="DG92" t="s">
         <v>32</v>
       </c>
-      <c r="DF92" t="s">
+      <c r="DH92" t="s">
         <v>32</v>
       </c>
-      <c r="DG92" t="s">
-        <v>8</v>
-      </c>
-      <c r="DH92" t="s">
-        <v>8</v>
-      </c>
       <c r="DI92" t="s">
         <v>8</v>
       </c>
@@ -3924,12 +3924,18 @@
         <v>8</v>
       </c>
       <c r="DK92" t="s">
-        <v>26</v>
+        <v>8</v>
       </c>
       <c r="DL92" t="s">
-        <v>10</v>
-      </c>
-      <c r="DR92" t="s">
+        <v>8</v>
+      </c>
+      <c r="DM92" t="s">
+        <v>26</v>
+      </c>
+      <c r="DN92" t="s">
+        <v>10</v>
+      </c>
+      <c r="DT92" t="s">
         <v>11</v>
       </c>
     </row>
@@ -3943,28 +3949,28 @@
       <c r="C93" t="s">
         <v>29</v>
       </c>
-      <c r="DB93" t="s">
-        <v>5</v>
-      </c>
-      <c r="DC93" t="s">
-        <v>6</v>
-      </c>
-      <c r="DF93" t="s">
+      <c r="DD93" t="s">
+        <v>5</v>
+      </c>
+      <c r="DE93" t="s">
+        <v>6</v>
+      </c>
+      <c r="DH93" t="s">
         <v>21</v>
       </c>
-      <c r="DL93" t="s">
-        <v>8</v>
-      </c>
-      <c r="DM93" t="s">
-        <v>8</v>
-      </c>
       <c r="DN93" t="s">
         <v>8</v>
       </c>
       <c r="DO93" t="s">
-        <v>10</v>
-      </c>
-      <c r="DS93" t="s">
+        <v>8</v>
+      </c>
+      <c r="DP93" t="s">
+        <v>8</v>
+      </c>
+      <c r="DQ93" t="s">
+        <v>10</v>
+      </c>
+      <c r="DU93" t="s">
         <v>11</v>
       </c>
     </row>
@@ -3978,31 +3984,31 @@
       <c r="C94" t="s">
         <v>31</v>
       </c>
-      <c r="DC94" t="s">
-        <v>5</v>
-      </c>
-      <c r="DD94" t="s">
-        <v>6</v>
-      </c>
-      <c r="DG94" t="s">
+      <c r="DE94" t="s">
+        <v>5</v>
+      </c>
+      <c r="DF94" t="s">
+        <v>6</v>
+      </c>
+      <c r="DI94" t="s">
         <v>30</v>
       </c>
-      <c r="DH94" t="s">
+      <c r="DJ94" t="s">
         <v>21</v>
       </c>
-      <c r="DO94" t="s">
-        <v>8</v>
-      </c>
-      <c r="DP94" t="s">
-        <v>26</v>
-      </c>
       <c r="DQ94" t="s">
-        <v>26</v>
+        <v>8</v>
       </c>
       <c r="DR94" t="s">
-        <v>10</v>
+        <v>26</v>
+      </c>
+      <c r="DS94" t="s">
+        <v>26</v>
       </c>
       <c r="DT94" t="s">
+        <v>10</v>
+      </c>
+      <c r="DV94" t="s">
         <v>11</v>
       </c>
     </row>
@@ -4016,19 +4022,19 @@
       <c r="C95" t="s">
         <v>33</v>
       </c>
-      <c r="DD95" t="s">
-        <v>5</v>
-      </c>
-      <c r="DE95" t="s">
-        <v>6</v>
-      </c>
-      <c r="DI95" t="s">
-        <v>8</v>
-      </c>
-      <c r="DJ95" t="s">
-        <v>10</v>
-      </c>
-      <c r="DU95" t="s">
+      <c r="DF95" t="s">
+        <v>5</v>
+      </c>
+      <c r="DG95" t="s">
+        <v>6</v>
+      </c>
+      <c r="DK95" t="s">
+        <v>8</v>
+      </c>
+      <c r="DL95" t="s">
+        <v>10</v>
+      </c>
+      <c r="DW95" t="s">
         <v>11</v>
       </c>
     </row>
@@ -4042,19 +4048,19 @@
       <c r="C96" t="s">
         <v>34</v>
       </c>
-      <c r="DE96" t="s">
-        <v>5</v>
-      </c>
-      <c r="DF96" t="s">
-        <v>6</v>
-      </c>
-      <c r="DJ96" t="s">
-        <v>8</v>
-      </c>
-      <c r="DK96" t="s">
-        <v>10</v>
-      </c>
-      <c r="DV96" t="s">
+      <c r="DG96" t="s">
+        <v>5</v>
+      </c>
+      <c r="DH96" t="s">
+        <v>6</v>
+      </c>
+      <c r="DL96" t="s">
+        <v>8</v>
+      </c>
+      <c r="DM96" t="s">
+        <v>10</v>
+      </c>
+      <c r="DX96" t="s">
         <v>11</v>
       </c>
     </row>
@@ -4068,28 +4074,28 @@
       <c r="C97" t="s">
         <v>35</v>
       </c>
-      <c r="DK97" t="s">
-        <v>5</v>
-      </c>
-      <c r="DL97" t="s">
-        <v>6</v>
-      </c>
       <c r="DM97" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="DN97" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="DO97" t="s">
         <v>8</v>
       </c>
       <c r="DP97" t="s">
-        <v>26</v>
+        <v>8</v>
       </c>
       <c r="DQ97" t="s">
-        <v>10</v>
-      </c>
-      <c r="DW97" t="s">
+        <v>8</v>
+      </c>
+      <c r="DR97" t="s">
+        <v>26</v>
+      </c>
+      <c r="DS97" t="s">
+        <v>10</v>
+      </c>
+      <c r="DY97" t="s">
         <v>11</v>
       </c>
     </row>
@@ -4103,28 +4109,28 @@
       <c r="C98" t="s">
         <v>36</v>
       </c>
-      <c r="DL98" t="s">
-        <v>5</v>
-      </c>
-      <c r="DM98" t="s">
-        <v>6</v>
-      </c>
       <c r="DN98" t="s">
+        <v>5</v>
+      </c>
+      <c r="DO98" t="s">
+        <v>6</v>
+      </c>
+      <c r="DP98" t="s">
         <v>21</v>
       </c>
-      <c r="DQ98" t="s">
-        <v>8</v>
-      </c>
-      <c r="DR98" t="s">
-        <v>8</v>
-      </c>
       <c r="DS98" t="s">
         <v>8</v>
       </c>
       <c r="DT98" t="s">
-        <v>10</v>
-      </c>
-      <c r="DX98" t="s">
+        <v>8</v>
+      </c>
+      <c r="DU98" t="s">
+        <v>8</v>
+      </c>
+      <c r="DV98" t="s">
+        <v>10</v>
+      </c>
+      <c r="DZ98" t="s">
         <v>11</v>
       </c>
     </row>
@@ -4138,19 +4144,19 @@
       <c r="C99" t="s">
         <v>37</v>
       </c>
-      <c r="DM99" t="s">
-        <v>5</v>
-      </c>
-      <c r="DN99" t="s">
-        <v>6</v>
-      </c>
       <c r="DO99" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="DP99" t="s">
-        <v>10</v>
-      </c>
-      <c r="DY99" t="s">
+        <v>6</v>
+      </c>
+      <c r="DQ99" t="s">
+        <v>8</v>
+      </c>
+      <c r="DR99" t="s">
+        <v>10</v>
+      </c>
+      <c r="EA99" t="s">
         <v>11</v>
       </c>
     </row>
@@ -4164,16 +4170,19 @@
       <c r="C100" t="s">
         <v>38</v>
       </c>
-      <c r="DN100" t="s">
-        <v>5</v>
-      </c>
       <c r="DP100" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="DQ100" t="s">
-        <v>10</v>
-      </c>
-      <c r="DZ100" t="s">
+        <v>6</v>
+      </c>
+      <c r="DR100" t="s">
+        <v>8</v>
+      </c>
+      <c r="DS100" t="s">
+        <v>10</v>
+      </c>
+      <c r="EB100" t="s">
         <v>11</v>
       </c>
     </row>
@@ -4187,46 +4196,22 @@
       <c r="C101" t="s">
         <v>39</v>
       </c>
-      <c r="DO101" t="s">
-        <v>5</v>
-      </c>
-      <c r="DP101" t="s">
-        <v>6</v>
-      </c>
-      <c r="DQ101" t="s">
-        <v>8</v>
-      </c>
-      <c r="DR101" t="s">
-        <v>26</v>
-      </c>
       <c r="DS101" t="s">
-        <v>26</v>
+        <v>5</v>
       </c>
       <c r="DT101" t="s">
-        <v>26</v>
+        <v>6</v>
       </c>
       <c r="DU101" t="s">
-        <v>26</v>
+        <v>8</v>
       </c>
       <c r="DV101" t="s">
         <v>26</v>
       </c>
       <c r="DW101" t="s">
-        <v>26</v>
-      </c>
-      <c r="DX101" t="s">
-        <v>26</v>
-      </c>
-      <c r="DY101" t="s">
-        <v>26</v>
-      </c>
-      <c r="DZ101" t="s">
-        <v>26</v>
-      </c>
-      <c r="EA101" t="s">
-        <v>26</v>
-      </c>
-      <c r="EB101" t="s">
+        <v>10</v>
+      </c>
+      <c r="EC101" t="s">
         <v>11</v>
       </c>
     </row>
@@ -4240,19 +4225,40 @@
       <c r="C102" t="s">
         <v>40</v>
       </c>
-      <c r="DP102" t="s">
-        <v>5</v>
-      </c>
-      <c r="DQ102" t="s">
-        <v>6</v>
-      </c>
-      <c r="DR102" t="s">
-        <v>8</v>
-      </c>
-      <c r="DS102" t="s">
-        <v>10</v>
+      <c r="DT102" t="s">
+        <v>5</v>
+      </c>
+      <c r="DU102" t="s">
+        <v>6</v>
+      </c>
+      <c r="DV102" t="s">
+        <v>8</v>
+      </c>
+      <c r="DW102" t="s">
+        <v>26</v>
+      </c>
+      <c r="DX102" t="s">
+        <v>26</v>
+      </c>
+      <c r="DY102" t="s">
+        <v>26</v>
+      </c>
+      <c r="DZ102" t="s">
+        <v>26</v>
+      </c>
+      <c r="EA102" t="s">
+        <v>26</v>
+      </c>
+      <c r="EB102" t="s">
+        <v>26</v>
       </c>
       <c r="EC102" t="s">
+        <v>26</v>
+      </c>
+      <c r="ED102" t="s">
+        <v>26</v>
+      </c>
+      <c r="EE102" t="s">
         <v>11</v>
       </c>
     </row>
@@ -4266,22 +4272,19 @@
       <c r="C103" t="s">
         <v>41</v>
       </c>
-      <c r="DQ103" t="s">
-        <v>5</v>
-      </c>
-      <c r="DR103" t="s">
-        <v>6</v>
-      </c>
-      <c r="DS103" t="s">
-        <v>8</v>
-      </c>
-      <c r="DT103" t="s">
-        <v>26</v>
-      </c>
       <c r="DU103" t="s">
-        <v>10</v>
-      </c>
-      <c r="ED103" t="s">
+        <v>5</v>
+      </c>
+      <c r="DV103" t="s">
+        <v>6</v>
+      </c>
+      <c r="DW103" t="s">
+        <v>8</v>
+      </c>
+      <c r="DX103" t="s">
+        <v>10</v>
+      </c>
+      <c r="EF103" t="s">
         <v>11</v>
       </c>
     </row>
@@ -4295,22 +4298,19 @@
       <c r="C104" t="s">
         <v>42</v>
       </c>
-      <c r="DR104" t="s">
-        <v>5</v>
-      </c>
-      <c r="DS104" t="s">
-        <v>6</v>
-      </c>
-      <c r="DT104" t="s">
-        <v>30</v>
-      </c>
-      <c r="DU104" t="s">
-        <v>8</v>
-      </c>
       <c r="DV104" t="s">
-        <v>10</v>
-      </c>
-      <c r="EE104" t="s">
+        <v>5</v>
+      </c>
+      <c r="DW104" t="s">
+        <v>6</v>
+      </c>
+      <c r="DX104" t="s">
+        <v>8</v>
+      </c>
+      <c r="DY104" t="s">
+        <v>10</v>
+      </c>
+      <c r="EG104" t="s">
         <v>11</v>
       </c>
     </row>
@@ -4324,19 +4324,19 @@
       <c r="C105" t="s">
         <v>43</v>
       </c>
-      <c r="DS105" t="s">
-        <v>5</v>
-      </c>
-      <c r="DT105" t="s">
-        <v>6</v>
-      </c>
-      <c r="DV105" t="s">
-        <v>8</v>
-      </c>
       <c r="DW105" t="s">
-        <v>10</v>
-      </c>
-      <c r="EF105" t="s">
+        <v>5</v>
+      </c>
+      <c r="DX105" t="s">
+        <v>6</v>
+      </c>
+      <c r="DY105" t="s">
+        <v>8</v>
+      </c>
+      <c r="DZ105" t="s">
+        <v>10</v>
+      </c>
+      <c r="EH105" t="s">
         <v>11</v>
       </c>
     </row>
@@ -4350,19 +4350,19 @@
       <c r="C106" t="s">
         <v>44</v>
       </c>
-      <c r="DT106" t="s">
-        <v>5</v>
-      </c>
-      <c r="DU106" t="s">
-        <v>6</v>
-      </c>
-      <c r="DW106" t="s">
-        <v>8</v>
-      </c>
       <c r="DX106" t="s">
-        <v>10</v>
-      </c>
-      <c r="EG106" t="s">
+        <v>5</v>
+      </c>
+      <c r="DY106" t="s">
+        <v>6</v>
+      </c>
+      <c r="DZ106" t="s">
+        <v>8</v>
+      </c>
+      <c r="EA106" t="s">
+        <v>10</v>
+      </c>
+      <c r="EI106" t="s">
         <v>11</v>
       </c>
     </row>
@@ -4376,19 +4376,19 @@
       <c r="C107" t="s">
         <v>45</v>
       </c>
-      <c r="DU107" t="s">
-        <v>5</v>
-      </c>
-      <c r="DV107" t="s">
-        <v>6</v>
-      </c>
-      <c r="DX107" t="s">
-        <v>8</v>
-      </c>
       <c r="DY107" t="s">
-        <v>10</v>
-      </c>
-      <c r="EH107" t="s">
+        <v>5</v>
+      </c>
+      <c r="DZ107" t="s">
+        <v>6</v>
+      </c>
+      <c r="EA107" t="s">
+        <v>8</v>
+      </c>
+      <c r="EB107" t="s">
+        <v>10</v>
+      </c>
+      <c r="EJ107" t="s">
         <v>11</v>
       </c>
     </row>
@@ -4402,19 +4402,19 @@
       <c r="C108" t="s">
         <v>46</v>
       </c>
-      <c r="DV108" t="s">
-        <v>5</v>
-      </c>
-      <c r="DW108" t="s">
-        <v>6</v>
-      </c>
-      <c r="DY108" t="s">
-        <v>8</v>
-      </c>
       <c r="DZ108" t="s">
-        <v>10</v>
-      </c>
-      <c r="EI108" t="s">
+        <v>5</v>
+      </c>
+      <c r="EA108" t="s">
+        <v>6</v>
+      </c>
+      <c r="EB108" t="s">
+        <v>8</v>
+      </c>
+      <c r="EC108" t="s">
+        <v>10</v>
+      </c>
+      <c r="EK108" t="s">
         <v>11</v>
       </c>
     </row>
@@ -4428,19 +4428,19 @@
       <c r="C109" t="s">
         <v>47</v>
       </c>
-      <c r="DW109" t="s">
-        <v>5</v>
-      </c>
-      <c r="DX109" t="s">
-        <v>6</v>
-      </c>
-      <c r="DZ109" t="s">
-        <v>8</v>
-      </c>
       <c r="EA109" t="s">
-        <v>10</v>
-      </c>
-      <c r="EJ109" t="s">
+        <v>5</v>
+      </c>
+      <c r="EB109" t="s">
+        <v>6</v>
+      </c>
+      <c r="EC109" t="s">
+        <v>8</v>
+      </c>
+      <c r="ED109" t="s">
+        <v>10</v>
+      </c>
+      <c r="EL109" t="s">
         <v>11</v>
       </c>
     </row>

</xml_diff>